<commit_message>
political_conservative annotated, finds added to other groups, grouping re-run
</commit_message>
<xml_diff>
--- a/0-assets/raw_data/main/3a-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
+++ b/0-assets/raw_data/main/3a-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
@@ -463,7 +463,7 @@
         <v>88</v>
       </c>
       <c r="C2" t="n">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -488,7 +488,7 @@
         <v>163</v>
       </c>
       <c r="C3" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -513,7 +513,7 @@
         <v>343</v>
       </c>
       <c r="C4" t="n">
-        <v>1283</v>
+        <v>1289</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -538,7 +538,7 @@
         <v>510</v>
       </c>
       <c r="C5" t="n">
-        <v>1442</v>
+        <v>1449</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -563,7 +563,7 @@
         <v>734</v>
       </c>
       <c r="C6" t="n">
-        <v>1816</v>
+        <v>1836</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -588,19 +588,19 @@
         <v>873</v>
       </c>
       <c r="C7" t="n">
-        <v>2276</v>
+        <v>2320</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8">
@@ -613,19 +613,19 @@
         <v>1590</v>
       </c>
       <c r="C8" t="n">
-        <v>2864</v>
+        <v>2913</v>
       </c>
       <c r="D8" t="n">
         <v>19</v>
       </c>
       <c r="E8" t="n">
-        <v>531</v>
+        <v>544</v>
       </c>
       <c r="F8" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G8" t="n">
-        <v>208</v>
+        <v>217</v>
       </c>
     </row>
     <row r="9">
@@ -638,19 +638,19 @@
         <v>1857</v>
       </c>
       <c r="C9" t="n">
-        <v>3244</v>
+        <v>3365</v>
       </c>
       <c r="D9" t="n">
         <v>25</v>
       </c>
       <c r="E9" t="n">
-        <v>774</v>
+        <v>798</v>
       </c>
       <c r="F9" t="n">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="G9" t="n">
-        <v>238</v>
+        <v>262</v>
       </c>
     </row>
     <row r="10">
@@ -663,7 +663,7 @@
         <v>43</v>
       </c>
       <c r="C10" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D10" t="n">
         <v>4</v>
@@ -688,10 +688,10 @@
         <v>108</v>
       </c>
       <c r="C11" t="n">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D11" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="E11" t="n">
         <v>15</v>
@@ -713,13 +713,13 @@
         <v>325</v>
       </c>
       <c r="C12" t="n">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D12" t="n">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F12" t="n">
         <v>46</v>
@@ -738,13 +738,13 @@
         <v>435</v>
       </c>
       <c r="C13" t="n">
-        <v>687</v>
+        <v>681</v>
       </c>
       <c r="D13" t="n">
-        <v>123</v>
+        <v>35</v>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F13" t="n">
         <v>82</v>
@@ -763,13 +763,13 @@
         <v>718</v>
       </c>
       <c r="C14" t="n">
-        <v>927</v>
+        <v>918</v>
       </c>
       <c r="D14" t="n">
-        <v>207</v>
+        <v>6</v>
       </c>
       <c r="E14" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F14" t="n">
         <v>197</v>
@@ -788,13 +788,13 @@
         <v>1183</v>
       </c>
       <c r="C15" t="n">
-        <v>1006</v>
+        <v>1002</v>
       </c>
       <c r="D15" t="n">
-        <v>328</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F15" t="n">
         <v>368</v>
@@ -813,13 +813,13 @@
         <v>1630</v>
       </c>
       <c r="C16" t="n">
-        <v>1180</v>
+        <v>1168</v>
       </c>
       <c r="D16" t="n">
-        <v>520</v>
+        <v>12</v>
       </c>
       <c r="E16" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F16" t="n">
         <v>575</v>
@@ -838,13 +838,13 @@
         <v>1887</v>
       </c>
       <c r="C17" t="n">
-        <v>1357</v>
+        <v>1349</v>
       </c>
       <c r="D17" t="n">
-        <v>675</v>
+        <v>11</v>
       </c>
       <c r="E17" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F17" t="n">
         <v>762</v>
@@ -863,10 +863,10 @@
         <v>2395</v>
       </c>
       <c r="C18" t="n">
-        <v>1590</v>
+        <v>1566</v>
       </c>
       <c r="D18" t="n">
-        <v>750</v>
+        <v>5</v>
       </c>
       <c r="E18" t="n">
         <v>38</v>
@@ -888,10 +888,10 @@
         <v>2124</v>
       </c>
       <c r="C19" t="n">
-        <v>1536</v>
+        <v>1507</v>
       </c>
       <c r="D19" t="n">
-        <v>613</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
         <v>44</v>
@@ -913,10 +913,10 @@
         <v>2134</v>
       </c>
       <c r="C20" t="n">
-        <v>1683</v>
+        <v>1643</v>
       </c>
       <c r="D20" t="n">
-        <v>592</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
         <v>42</v>
@@ -941,7 +941,7 @@
         <v>1738</v>
       </c>
       <c r="D21" t="n">
-        <v>515</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
         <v>41</v>
@@ -963,10 +963,10 @@
         <v>1592</v>
       </c>
       <c r="C22" t="n">
-        <v>1914</v>
+        <v>1911</v>
       </c>
       <c r="D22" t="n">
-        <v>552</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
         <v>51</v>
@@ -988,10 +988,10 @@
         <v>1424</v>
       </c>
       <c r="C23" t="n">
-        <v>1863</v>
+        <v>1826</v>
       </c>
       <c r="D23" t="n">
-        <v>472</v>
+        <v>4</v>
       </c>
       <c r="E23" t="n">
         <v>133</v>
@@ -1013,13 +1013,13 @@
         <v>1496</v>
       </c>
       <c r="C24" t="n">
-        <v>1730</v>
+        <v>1711</v>
       </c>
       <c r="D24" t="n">
-        <v>469</v>
+        <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F24" t="n">
         <v>750</v>
@@ -1038,10 +1038,10 @@
         <v>1207</v>
       </c>
       <c r="C25" t="n">
-        <v>1732</v>
+        <v>1688</v>
       </c>
       <c r="D25" t="n">
-        <v>400</v>
+        <v>11</v>
       </c>
       <c r="E25" t="n">
         <v>345</v>
@@ -1063,10 +1063,10 @@
         <v>1367</v>
       </c>
       <c r="C26" t="n">
-        <v>1729</v>
+        <v>1713</v>
       </c>
       <c r="D26" t="n">
-        <v>559</v>
+        <v>28</v>
       </c>
       <c r="E26" t="n">
         <v>742</v>
@@ -1088,10 +1088,10 @@
         <v>1291</v>
       </c>
       <c r="C27" t="n">
-        <v>1883</v>
+        <v>1861</v>
       </c>
       <c r="D27" t="n">
-        <v>568</v>
+        <v>14</v>
       </c>
       <c r="E27" t="n">
         <v>451</v>
@@ -1113,10 +1113,10 @@
         <v>1320</v>
       </c>
       <c r="C28" t="n">
-        <v>1793</v>
+        <v>1782</v>
       </c>
       <c r="D28" t="n">
-        <v>595</v>
+        <v>7</v>
       </c>
       <c r="E28" t="n">
         <v>142</v>
@@ -1138,13 +1138,13 @@
         <v>1198</v>
       </c>
       <c r="C29" t="n">
-        <v>1860</v>
+        <v>1844</v>
       </c>
       <c r="D29" t="n">
-        <v>770</v>
+        <v>12</v>
       </c>
       <c r="E29" t="n">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F29" t="n">
         <v>917</v>
@@ -1163,10 +1163,10 @@
         <v>1067</v>
       </c>
       <c r="C30" t="n">
-        <v>1751</v>
+        <v>1734</v>
       </c>
       <c r="D30" t="n">
-        <v>1003</v>
+        <v>15</v>
       </c>
       <c r="E30" t="n">
         <v>557</v>
@@ -1188,13 +1188,13 @@
         <v>919</v>
       </c>
       <c r="C31" t="n">
-        <v>1739</v>
+        <v>1721</v>
       </c>
       <c r="D31" t="n">
-        <v>695</v>
+        <v>18</v>
       </c>
       <c r="E31" t="n">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="F31" t="n">
         <v>962</v>
@@ -1213,13 +1213,13 @@
         <v>852</v>
       </c>
       <c r="C32" t="n">
-        <v>1635</v>
+        <v>1620</v>
       </c>
       <c r="D32" t="n">
-        <v>575</v>
+        <v>15</v>
       </c>
       <c r="E32" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="F32" t="n">
         <v>933</v>
@@ -1238,10 +1238,10 @@
         <v>818</v>
       </c>
       <c r="C33" t="n">
-        <v>1446</v>
+        <v>1410</v>
       </c>
       <c r="D33" t="n">
-        <v>609</v>
+        <v>13</v>
       </c>
       <c r="E33" t="n">
         <v>823</v>
@@ -1263,10 +1263,10 @@
         <v>793</v>
       </c>
       <c r="C34" t="n">
-        <v>1399</v>
+        <v>1391</v>
       </c>
       <c r="D34" t="n">
-        <v>664</v>
+        <v>32</v>
       </c>
       <c r="E34" t="n">
         <v>900</v>
@@ -1288,10 +1288,10 @@
         <v>930</v>
       </c>
       <c r="C35" t="n">
-        <v>1545</v>
+        <v>1536</v>
       </c>
       <c r="D35" t="n">
-        <v>841</v>
+        <v>44</v>
       </c>
       <c r="E35" t="n">
         <v>977</v>
@@ -1313,10 +1313,10 @@
         <v>848</v>
       </c>
       <c r="C36" t="n">
-        <v>1243</v>
+        <v>1223</v>
       </c>
       <c r="D36" t="n">
-        <v>886</v>
+        <v>45</v>
       </c>
       <c r="E36" t="n">
         <v>1200</v>
@@ -1338,10 +1338,10 @@
         <v>879</v>
       </c>
       <c r="C37" t="n">
-        <v>1078</v>
+        <v>1073</v>
       </c>
       <c r="D37" t="n">
-        <v>875</v>
+        <v>65</v>
       </c>
       <c r="E37" t="n">
         <v>1168</v>
@@ -1363,10 +1363,10 @@
         <v>920</v>
       </c>
       <c r="C38" t="n">
-        <v>1101</v>
+        <v>1091</v>
       </c>
       <c r="D38" t="n">
-        <v>746</v>
+        <v>47</v>
       </c>
       <c r="E38" t="n">
         <v>1186</v>
@@ -1388,10 +1388,10 @@
         <v>882</v>
       </c>
       <c r="C39" t="n">
-        <v>2762</v>
+        <v>2755</v>
       </c>
       <c r="D39" t="n">
-        <v>632</v>
+        <v>49</v>
       </c>
       <c r="E39" t="n">
         <v>928</v>
@@ -1413,10 +1413,10 @@
         <v>945</v>
       </c>
       <c r="C40" t="n">
-        <v>3530</v>
+        <v>3521</v>
       </c>
       <c r="D40" t="n">
-        <v>651</v>
+        <v>78</v>
       </c>
       <c r="E40" t="n">
         <v>1045</v>
@@ -1438,10 +1438,10 @@
         <v>1209</v>
       </c>
       <c r="C41" t="n">
-        <v>2718</v>
+        <v>2715</v>
       </c>
       <c r="D41" t="n">
-        <v>700</v>
+        <v>104</v>
       </c>
       <c r="E41" t="n">
         <v>1012</v>
@@ -1463,16 +1463,16 @@
         <v>1153</v>
       </c>
       <c r="C42" t="n">
-        <v>2210</v>
+        <v>2206</v>
       </c>
       <c r="D42" t="n">
-        <v>729</v>
+        <v>133</v>
       </c>
       <c r="E42" t="n">
         <v>1032</v>
       </c>
       <c r="F42" t="n">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="G42" t="n">
         <v>557</v>
@@ -1488,10 +1488,10 @@
         <v>1201</v>
       </c>
       <c r="C43" t="n">
-        <v>2340</v>
+        <v>2336</v>
       </c>
       <c r="D43" t="n">
-        <v>910</v>
+        <v>199</v>
       </c>
       <c r="E43" t="n">
         <v>836</v>
@@ -1513,10 +1513,10 @@
         <v>1227</v>
       </c>
       <c r="C44" t="n">
-        <v>2351</v>
+        <v>2350</v>
       </c>
       <c r="D44" t="n">
-        <v>904</v>
+        <v>242</v>
       </c>
       <c r="E44" t="n">
         <v>922</v>
@@ -1538,10 +1538,10 @@
         <v>1010</v>
       </c>
       <c r="C45" t="n">
-        <v>1713</v>
+        <v>1703</v>
       </c>
       <c r="D45" t="n">
-        <v>887</v>
+        <v>273</v>
       </c>
       <c r="E45" t="n">
         <v>1060</v>
@@ -1550,7 +1550,7 @@
         <v>495</v>
       </c>
       <c r="G45" t="n">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="46">
@@ -1563,10 +1563,10 @@
         <v>908</v>
       </c>
       <c r="C46" t="n">
-        <v>2278</v>
+        <v>2256</v>
       </c>
       <c r="D46" t="n">
-        <v>583</v>
+        <v>141</v>
       </c>
       <c r="E46" t="n">
         <v>917</v>
@@ -1588,10 +1588,10 @@
         <v>1018</v>
       </c>
       <c r="C47" t="n">
-        <v>2433</v>
+        <v>2415</v>
       </c>
       <c r="D47" t="n">
-        <v>527</v>
+        <v>129</v>
       </c>
       <c r="E47" t="n">
         <v>682</v>
@@ -1613,10 +1613,10 @@
         <v>1012</v>
       </c>
       <c r="C48" t="n">
-        <v>2963</v>
+        <v>2922</v>
       </c>
       <c r="D48" t="n">
-        <v>595</v>
+        <v>108</v>
       </c>
       <c r="E48" t="n">
         <v>685</v>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-10T10:57:50</t>
+          <t>2026-10-10T17:49:44</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0h 06m 51s</t>
+          <t>0h 06m 34s</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0h 06m 53s</t>
+          <t>0h 06m 35s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-ran grouping for statistics
</commit_message>
<xml_diff>
--- a/0-assets/raw_data/main/3a-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
+++ b/0-assets/raw_data/main/3a-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
@@ -675,7 +675,7 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>90</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -700,7 +700,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>63</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -725,7 +725,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -747,10 +747,10 @@
         <v>15</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>52</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -772,10 +772,10 @@
         <v>21</v>
       </c>
       <c r="F14" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>68</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -800,7 +800,7 @@
         <v>50</v>
       </c>
       <c r="G15" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -822,10 +822,10 @@
         <v>23</v>
       </c>
       <c r="F16" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G16" t="n">
-        <v>82</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17">
@@ -847,10 +847,10 @@
         <v>19</v>
       </c>
       <c r="F17" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G17" t="n">
-        <v>79</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18">
@@ -875,7 +875,7 @@
         <v>118</v>
       </c>
       <c r="G18" t="n">
-        <v>95</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19">
@@ -897,10 +897,10 @@
         <v>42</v>
       </c>
       <c r="F19" t="n">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G19" t="n">
-        <v>85</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2138</v>
+        <v>2139</v>
       </c>
       <c r="C20" t="n">
         <v>1662</v>
@@ -922,10 +922,10 @@
         <v>37</v>
       </c>
       <c r="F20" t="n">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="G20" t="n">
-        <v>126</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21">
@@ -947,10 +947,10 @@
         <v>36</v>
       </c>
       <c r="F21" t="n">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="G21" t="n">
-        <v>121</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22">
@@ -972,10 +972,10 @@
         <v>46</v>
       </c>
       <c r="F22" t="n">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="G22" t="n">
-        <v>162</v>
+        <v>103</v>
       </c>
     </row>
     <row r="23">
@@ -997,10 +997,10 @@
         <v>73</v>
       </c>
       <c r="F23" t="n">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="G23" t="n">
-        <v>180</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24">
@@ -1022,10 +1022,10 @@
         <v>170</v>
       </c>
       <c r="F24" t="n">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="G24" t="n">
-        <v>202</v>
+        <v>130</v>
       </c>
     </row>
     <row r="25">
@@ -1044,13 +1044,13 @@
         <v>11</v>
       </c>
       <c r="E25" t="n">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F25" t="n">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="G25" t="n">
-        <v>228</v>
+        <v>143</v>
       </c>
     </row>
     <row r="26">
@@ -1072,10 +1072,10 @@
         <v>404</v>
       </c>
       <c r="F26" t="n">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="G26" t="n">
-        <v>213</v>
+        <v>123</v>
       </c>
     </row>
     <row r="27">
@@ -1094,13 +1094,13 @@
         <v>14</v>
       </c>
       <c r="E27" t="n">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F27" t="n">
+        <v>198</v>
+      </c>
+      <c r="G27" t="n">
         <v>195</v>
-      </c>
-      <c r="G27" t="n">
-        <v>311</v>
       </c>
     </row>
     <row r="28">
@@ -1119,13 +1119,13 @@
         <v>7</v>
       </c>
       <c r="E28" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F28" t="n">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="G28" t="n">
-        <v>291</v>
+        <v>192</v>
       </c>
     </row>
     <row r="29">
@@ -1147,10 +1147,10 @@
         <v>94</v>
       </c>
       <c r="F29" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G29" t="n">
-        <v>311</v>
+        <v>211</v>
       </c>
     </row>
     <row r="30">
@@ -1172,10 +1172,10 @@
         <v>124</v>
       </c>
       <c r="F30" t="n">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G30" t="n">
-        <v>356</v>
+        <v>212</v>
       </c>
     </row>
     <row r="31">
@@ -1197,10 +1197,10 @@
         <v>114</v>
       </c>
       <c r="F31" t="n">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="G31" t="n">
-        <v>415</v>
+        <v>254</v>
       </c>
     </row>
     <row r="32">
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>862</v>
+        <v>865</v>
       </c>
       <c r="C32" t="n">
         <v>1639</v>
@@ -1222,10 +1222,10 @@
         <v>128</v>
       </c>
       <c r="F32" t="n">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="G32" t="n">
-        <v>427</v>
+        <v>273</v>
       </c>
     </row>
     <row r="33">
@@ -1247,10 +1247,10 @@
         <v>179</v>
       </c>
       <c r="F33" t="n">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G33" t="n">
-        <v>445</v>
+        <v>276</v>
       </c>
     </row>
     <row r="34">
@@ -1275,7 +1275,7 @@
         <v>201</v>
       </c>
       <c r="G34" t="n">
-        <v>441</v>
+        <v>232</v>
       </c>
     </row>
     <row r="35">
@@ -1297,10 +1297,10 @@
         <v>173</v>
       </c>
       <c r="F35" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="G35" t="n">
-        <v>525</v>
+        <v>326</v>
       </c>
     </row>
     <row r="36">
@@ -1322,10 +1322,10 @@
         <v>169</v>
       </c>
       <c r="F36" t="n">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="G36" t="n">
-        <v>425</v>
+        <v>275</v>
       </c>
     </row>
     <row r="37">
@@ -1338,7 +1338,7 @@
         <v>886</v>
       </c>
       <c r="C37" t="n">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="D37" t="n">
         <v>67</v>
@@ -1347,10 +1347,10 @@
         <v>196</v>
       </c>
       <c r="F37" t="n">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="G37" t="n">
-        <v>366</v>
+        <v>208</v>
       </c>
     </row>
     <row r="38">
@@ -1360,10 +1360,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="C38" t="n">
-        <v>1182</v>
+        <v>1185</v>
       </c>
       <c r="D38" t="n">
         <v>49</v>
@@ -1375,7 +1375,7 @@
         <v>274</v>
       </c>
       <c r="G38" t="n">
-        <v>404</v>
+        <v>227</v>
       </c>
     </row>
     <row r="39">
@@ -1388,7 +1388,7 @@
         <v>890</v>
       </c>
       <c r="C39" t="n">
-        <v>2855</v>
+        <v>2856</v>
       </c>
       <c r="D39" t="n">
         <v>50</v>
@@ -1397,10 +1397,10 @@
         <v>252</v>
       </c>
       <c r="F39" t="n">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="G39" t="n">
-        <v>357</v>
+        <v>196</v>
       </c>
     </row>
     <row r="40">
@@ -1410,10 +1410,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="C40" t="n">
-        <v>3633</v>
+        <v>3642</v>
       </c>
       <c r="D40" t="n">
         <v>80</v>
@@ -1422,10 +1422,10 @@
         <v>253</v>
       </c>
       <c r="F40" t="n">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="G40" t="n">
-        <v>411</v>
+        <v>242</v>
       </c>
     </row>
     <row r="41">
@@ -1435,22 +1435,22 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1220</v>
+        <v>1222</v>
       </c>
       <c r="C41" t="n">
-        <v>2763</v>
+        <v>2783</v>
       </c>
       <c r="D41" t="n">
         <v>104</v>
       </c>
       <c r="E41" t="n">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="F41" t="n">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="G41" t="n">
-        <v>592</v>
+        <v>333</v>
       </c>
     </row>
     <row r="42">
@@ -1460,10 +1460,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1155</v>
+        <v>1160</v>
       </c>
       <c r="C42" t="n">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="D42" t="n">
         <v>133</v>
@@ -1472,10 +1472,10 @@
         <v>389</v>
       </c>
       <c r="F42" t="n">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="G42" t="n">
-        <v>557</v>
+        <v>244</v>
       </c>
     </row>
     <row r="43">
@@ -1497,10 +1497,10 @@
         <v>283</v>
       </c>
       <c r="F43" t="n">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="G43" t="n">
-        <v>497</v>
+        <v>206</v>
       </c>
     </row>
     <row r="44">
@@ -1510,10 +1510,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="C44" t="n">
-        <v>2354</v>
+        <v>2355</v>
       </c>
       <c r="D44" t="n">
         <v>243</v>
@@ -1522,10 +1522,10 @@
         <v>319</v>
       </c>
       <c r="F44" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G44" t="n">
-        <v>467</v>
+        <v>233</v>
       </c>
     </row>
     <row r="45">
@@ -1535,10 +1535,10 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1010</v>
+        <v>1012</v>
       </c>
       <c r="C45" t="n">
-        <v>1710</v>
+        <v>1712</v>
       </c>
       <c r="D45" t="n">
         <v>275</v>
@@ -1547,10 +1547,10 @@
         <v>314</v>
       </c>
       <c r="F45" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G45" t="n">
-        <v>471</v>
+        <v>211</v>
       </c>
     </row>
     <row r="46">
@@ -1575,7 +1575,7 @@
         <v>26</v>
       </c>
       <c r="G46" t="n">
-        <v>580</v>
+        <v>182</v>
       </c>
     </row>
     <row r="47">
@@ -1597,10 +1597,10 @@
         <v>300</v>
       </c>
       <c r="F47" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="G47" t="n">
-        <v>786</v>
+        <v>239</v>
       </c>
     </row>
     <row r="48">
@@ -1622,10 +1622,10 @@
         <v>316</v>
       </c>
       <c r="F48" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G48" t="n">
-        <v>919</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-13T10:41:54</t>
+          <t>2026-10-13T22:09:53</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0h 08m 14s</t>
+          <t>0h 10m 16s</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0h 08m 17s</t>
+          <t>0h 10m 19s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
gender_female change fixed; pipeline re-run
</commit_message>
<xml_diff>
--- a/0-assets/raw_data/main/3a-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
+++ b/0-assets/raw_data/main/3a-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
@@ -429,7 +429,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>gender_female_or_diverse</t>
+          <t>gender_female</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -475,7 +475,7 @@
         <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>19</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3">
@@ -500,7 +500,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>21</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4">
@@ -525,7 +525,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>42</v>
+        <v>371</v>
       </c>
     </row>
     <row r="5">
@@ -550,7 +550,7 @@
         <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>97</v>
+        <v>520</v>
       </c>
     </row>
     <row r="6">
@@ -575,7 +575,7 @@
         <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>122</v>
+        <v>617</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +600,7 @@
         <v>3</v>
       </c>
       <c r="G7" t="n">
-        <v>106</v>
+        <v>770</v>
       </c>
     </row>
     <row r="8">
@@ -625,7 +625,7 @@
         <v>35</v>
       </c>
       <c r="G8" t="n">
-        <v>226</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +650,7 @@
         <v>42</v>
       </c>
       <c r="G9" t="n">
-        <v>263</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="10">
@@ -663,7 +663,7 @@
         <v>43</v>
       </c>
       <c r="C10" t="n">
-        <v>96</v>
+        <v>40</v>
       </c>
       <c r="D10" t="n">
         <v>4</v>
@@ -675,7 +675,7 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
@@ -688,7 +688,7 @@
         <v>108</v>
       </c>
       <c r="C11" t="n">
-        <v>196</v>
+        <v>148</v>
       </c>
       <c r="D11" t="n">
         <v>7</v>
@@ -700,7 +700,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -713,7 +713,7 @@
         <v>323</v>
       </c>
       <c r="C12" t="n">
-        <v>503</v>
+        <v>456</v>
       </c>
       <c r="D12" t="n">
         <v>15</v>
@@ -725,7 +725,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -738,7 +738,7 @@
         <v>435</v>
       </c>
       <c r="C13" t="n">
-        <v>680</v>
+        <v>615</v>
       </c>
       <c r="D13" t="n">
         <v>31</v>
@@ -750,7 +750,7 @@
         <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14">
@@ -763,7 +763,7 @@
         <v>721</v>
       </c>
       <c r="C14" t="n">
-        <v>918</v>
+        <v>855</v>
       </c>
       <c r="D14" t="n">
         <v>6</v>
@@ -775,7 +775,7 @@
         <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         <v>1190</v>
       </c>
       <c r="C15" t="n">
-        <v>999</v>
+        <v>914</v>
       </c>
       <c r="D15" t="n">
         <v>8</v>
@@ -800,7 +800,7 @@
         <v>50</v>
       </c>
       <c r="G15" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16">
@@ -813,7 +813,7 @@
         <v>1637</v>
       </c>
       <c r="C16" t="n">
-        <v>1176</v>
+        <v>1014</v>
       </c>
       <c r="D16" t="n">
         <v>12</v>
@@ -825,7 +825,7 @@
         <v>64</v>
       </c>
       <c r="G16" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17">
@@ -838,7 +838,7 @@
         <v>1892</v>
       </c>
       <c r="C17" t="n">
-        <v>1360</v>
+        <v>1188</v>
       </c>
       <c r="D17" t="n">
         <v>10</v>
@@ -850,7 +850,7 @@
         <v>97</v>
       </c>
       <c r="G17" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18">
@@ -863,7 +863,7 @@
         <v>2400</v>
       </c>
       <c r="C18" t="n">
-        <v>1578</v>
+        <v>1382</v>
       </c>
       <c r="D18" t="n">
         <v>5</v>
@@ -875,7 +875,7 @@
         <v>118</v>
       </c>
       <c r="G18" t="n">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19">
@@ -888,7 +888,7 @@
         <v>2118</v>
       </c>
       <c r="C19" t="n">
-        <v>1511</v>
+        <v>1355</v>
       </c>
       <c r="D19" t="n">
         <v>3</v>
@@ -900,7 +900,7 @@
         <v>145</v>
       </c>
       <c r="G19" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20">
@@ -913,7 +913,7 @@
         <v>2133</v>
       </c>
       <c r="C20" t="n">
-        <v>1662</v>
+        <v>1377</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
@@ -925,7 +925,7 @@
         <v>243</v>
       </c>
       <c r="G20" t="n">
-        <v>69</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21">
@@ -938,7 +938,7 @@
         <v>1805</v>
       </c>
       <c r="C21" t="n">
-        <v>1757</v>
+        <v>1409</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -950,7 +950,7 @@
         <v>230</v>
       </c>
       <c r="G21" t="n">
-        <v>72</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22">
@@ -963,7 +963,7 @@
         <v>1635</v>
       </c>
       <c r="C22" t="n">
-        <v>1917</v>
+        <v>1458</v>
       </c>
       <c r="D22" t="n">
         <v>4</v>
@@ -975,7 +975,7 @@
         <v>252</v>
       </c>
       <c r="G22" t="n">
-        <v>103</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23">
@@ -988,7 +988,7 @@
         <v>1428</v>
       </c>
       <c r="C23" t="n">
-        <v>1834</v>
+        <v>1320</v>
       </c>
       <c r="D23" t="n">
         <v>4</v>
@@ -1000,7 +1000,7 @@
         <v>250</v>
       </c>
       <c r="G23" t="n">
-        <v>120</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24">
@@ -1013,7 +1013,7 @@
         <v>1502</v>
       </c>
       <c r="C24" t="n">
-        <v>1732</v>
+        <v>1257</v>
       </c>
       <c r="D24" t="n">
         <v>9</v>
@@ -1025,7 +1025,7 @@
         <v>233</v>
       </c>
       <c r="G24" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
     </row>
     <row r="25">
@@ -1038,7 +1038,7 @@
         <v>1212</v>
       </c>
       <c r="C25" t="n">
-        <v>1716</v>
+        <v>1095</v>
       </c>
       <c r="D25" t="n">
         <v>11</v>
@@ -1050,7 +1050,7 @@
         <v>284</v>
       </c>
       <c r="G25" t="n">
-        <v>143</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26">
@@ -1063,7 +1063,7 @@
         <v>1367</v>
       </c>
       <c r="C26" t="n">
-        <v>1746</v>
+        <v>1215</v>
       </c>
       <c r="D26" t="n">
         <v>28</v>
@@ -1075,7 +1075,7 @@
         <v>258</v>
       </c>
       <c r="G26" t="n">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="27">
@@ -1088,7 +1088,7 @@
         <v>1287</v>
       </c>
       <c r="C27" t="n">
-        <v>1871</v>
+        <v>1176</v>
       </c>
       <c r="D27" t="n">
         <v>14</v>
@@ -1100,7 +1100,7 @@
         <v>198</v>
       </c>
       <c r="G27" t="n">
-        <v>195</v>
+        <v>201</v>
       </c>
     </row>
     <row r="28">
@@ -1113,7 +1113,7 @@
         <v>1333</v>
       </c>
       <c r="C28" t="n">
-        <v>1822</v>
+        <v>1084</v>
       </c>
       <c r="D28" t="n">
         <v>7</v>
@@ -1125,7 +1125,7 @@
         <v>199</v>
       </c>
       <c r="G28" t="n">
-        <v>192</v>
+        <v>219</v>
       </c>
     </row>
     <row r="29">
@@ -1138,7 +1138,7 @@
         <v>1201</v>
       </c>
       <c r="C29" t="n">
-        <v>1887</v>
+        <v>1107</v>
       </c>
       <c r="D29" t="n">
         <v>11</v>
@@ -1150,7 +1150,7 @@
         <v>235</v>
       </c>
       <c r="G29" t="n">
-        <v>211</v>
+        <v>228</v>
       </c>
     </row>
     <row r="30">
@@ -1163,7 +1163,7 @@
         <v>1070</v>
       </c>
       <c r="C30" t="n">
-        <v>1774</v>
+        <v>987</v>
       </c>
       <c r="D30" t="n">
         <v>15</v>
@@ -1175,7 +1175,7 @@
         <v>212</v>
       </c>
       <c r="G30" t="n">
-        <v>212</v>
+        <v>226</v>
       </c>
     </row>
     <row r="31">
@@ -1188,7 +1188,7 @@
         <v>913</v>
       </c>
       <c r="C31" t="n">
-        <v>1746</v>
+        <v>907</v>
       </c>
       <c r="D31" t="n">
         <v>16</v>
@@ -1200,7 +1200,7 @@
         <v>227</v>
       </c>
       <c r="G31" t="n">
-        <v>254</v>
+        <v>268</v>
       </c>
     </row>
     <row r="32">
@@ -1213,7 +1213,7 @@
         <v>857</v>
       </c>
       <c r="C32" t="n">
-        <v>1637</v>
+        <v>803</v>
       </c>
       <c r="D32" t="n">
         <v>16</v>
@@ -1225,7 +1225,7 @@
         <v>231</v>
       </c>
       <c r="G32" t="n">
-        <v>273</v>
+        <v>299</v>
       </c>
     </row>
     <row r="33">
@@ -1238,7 +1238,7 @@
         <v>818</v>
       </c>
       <c r="C33" t="n">
-        <v>1464</v>
+        <v>750</v>
       </c>
       <c r="D33" t="n">
         <v>14</v>
@@ -1250,7 +1250,7 @@
         <v>239</v>
       </c>
       <c r="G33" t="n">
-        <v>276</v>
+        <v>301</v>
       </c>
     </row>
     <row r="34">
@@ -1263,7 +1263,7 @@
         <v>792</v>
       </c>
       <c r="C34" t="n">
-        <v>1418</v>
+        <v>681</v>
       </c>
       <c r="D34" t="n">
         <v>33</v>
@@ -1275,7 +1275,7 @@
         <v>201</v>
       </c>
       <c r="G34" t="n">
-        <v>232</v>
+        <v>257</v>
       </c>
     </row>
     <row r="35">
@@ -1288,7 +1288,7 @@
         <v>941</v>
       </c>
       <c r="C35" t="n">
-        <v>1572</v>
+        <v>763</v>
       </c>
       <c r="D35" t="n">
         <v>45</v>
@@ -1300,7 +1300,7 @@
         <v>286</v>
       </c>
       <c r="G35" t="n">
-        <v>326</v>
+        <v>361</v>
       </c>
     </row>
     <row r="36">
@@ -1313,7 +1313,7 @@
         <v>850</v>
       </c>
       <c r="C36" t="n">
-        <v>1291</v>
+        <v>678</v>
       </c>
       <c r="D36" t="n">
         <v>49</v>
@@ -1325,7 +1325,7 @@
         <v>318</v>
       </c>
       <c r="G36" t="n">
-        <v>275</v>
+        <v>292</v>
       </c>
     </row>
     <row r="37">
@@ -1338,7 +1338,7 @@
         <v>885</v>
       </c>
       <c r="C37" t="n">
-        <v>1148</v>
+        <v>697</v>
       </c>
       <c r="D37" t="n">
         <v>67</v>
@@ -1350,7 +1350,7 @@
         <v>293</v>
       </c>
       <c r="G37" t="n">
-        <v>208</v>
+        <v>228</v>
       </c>
     </row>
     <row r="38">
@@ -1363,7 +1363,7 @@
         <v>934</v>
       </c>
       <c r="C38" t="n">
-        <v>1185</v>
+        <v>774</v>
       </c>
       <c r="D38" t="n">
         <v>49</v>
@@ -1375,7 +1375,7 @@
         <v>274</v>
       </c>
       <c r="G38" t="n">
-        <v>227</v>
+        <v>258</v>
       </c>
     </row>
     <row r="39">
@@ -1388,7 +1388,7 @@
         <v>890</v>
       </c>
       <c r="C39" t="n">
-        <v>2853</v>
+        <v>2485</v>
       </c>
       <c r="D39" t="n">
         <v>50</v>
@@ -1400,7 +1400,7 @@
         <v>317</v>
       </c>
       <c r="G39" t="n">
-        <v>196</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40">
@@ -1413,7 +1413,7 @@
         <v>952</v>
       </c>
       <c r="C40" t="n">
-        <v>3640</v>
+        <v>3273</v>
       </c>
       <c r="D40" t="n">
         <v>79</v>
@@ -1425,7 +1425,7 @@
         <v>293</v>
       </c>
       <c r="G40" t="n">
-        <v>242</v>
+        <v>275</v>
       </c>
     </row>
     <row r="41">
@@ -1438,7 +1438,7 @@
         <v>1215</v>
       </c>
       <c r="C41" t="n">
-        <v>2780</v>
+        <v>2411</v>
       </c>
       <c r="D41" t="n">
         <v>104</v>
@@ -1450,7 +1450,7 @@
         <v>237</v>
       </c>
       <c r="G41" t="n">
-        <v>333</v>
+        <v>363</v>
       </c>
     </row>
     <row r="42">
@@ -1463,7 +1463,7 @@
         <v>1139</v>
       </c>
       <c r="C42" t="n">
-        <v>2249</v>
+        <v>1915</v>
       </c>
       <c r="D42" t="n">
         <v>133</v>
@@ -1475,7 +1475,7 @@
         <v>243</v>
       </c>
       <c r="G42" t="n">
-        <v>244</v>
+        <v>294</v>
       </c>
     </row>
     <row r="43">
@@ -1488,7 +1488,7 @@
         <v>1188</v>
       </c>
       <c r="C43" t="n">
-        <v>2337</v>
+        <v>1987</v>
       </c>
       <c r="D43" t="n">
         <v>203</v>
@@ -1500,7 +1500,7 @@
         <v>87</v>
       </c>
       <c r="G43" t="n">
-        <v>206</v>
+        <v>268</v>
       </c>
     </row>
     <row r="44">
@@ -1513,7 +1513,7 @@
         <v>1222</v>
       </c>
       <c r="C44" t="n">
-        <v>2349</v>
+        <v>1897</v>
       </c>
       <c r="D44" t="n">
         <v>242</v>
@@ -1525,7 +1525,7 @@
         <v>45</v>
       </c>
       <c r="G44" t="n">
-        <v>233</v>
+        <v>333</v>
       </c>
     </row>
     <row r="45">
@@ -1538,7 +1538,7 @@
         <v>1011</v>
       </c>
       <c r="C45" t="n">
-        <v>1702</v>
+        <v>1336</v>
       </c>
       <c r="D45" t="n">
         <v>275</v>
@@ -1550,7 +1550,7 @@
         <v>38</v>
       </c>
       <c r="G45" t="n">
-        <v>211</v>
+        <v>300</v>
       </c>
     </row>
     <row r="46">
@@ -1563,7 +1563,7 @@
         <v>903</v>
       </c>
       <c r="C46" t="n">
-        <v>2253</v>
+        <v>1863</v>
       </c>
       <c r="D46" t="n">
         <v>144</v>
@@ -1575,7 +1575,7 @@
         <v>26</v>
       </c>
       <c r="G46" t="n">
-        <v>182</v>
+        <v>287</v>
       </c>
     </row>
     <row r="47">
@@ -1588,7 +1588,7 @@
         <v>1010</v>
       </c>
       <c r="C47" t="n">
-        <v>2408</v>
+        <v>1823</v>
       </c>
       <c r="D47" t="n">
         <v>135</v>
@@ -1600,7 +1600,7 @@
         <v>36</v>
       </c>
       <c r="G47" t="n">
-        <v>239</v>
+        <v>411</v>
       </c>
     </row>
     <row r="48">
@@ -1613,7 +1613,7 @@
         <v>1002</v>
       </c>
       <c r="C48" t="n">
-        <v>2918</v>
+        <v>2200</v>
       </c>
       <c r="D48" t="n">
         <v>111</v>
@@ -1625,7 +1625,7 @@
         <v>46</v>
       </c>
       <c r="G48" t="n">
-        <v>268</v>
+        <v>442</v>
       </c>
     </row>
   </sheetData>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-15T18:30:57</t>
+          <t>2026-10-15T23:03:23</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0h 15m 20s</t>
+          <t>0h 16m 35s</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0h 15m 27s</t>
+          <t>0h 16m 40s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Claude Opus Extra high effort corrections
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/0-assets/raw_data/main/3a-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
+++ b/0-assets/raw_data/main/3a-grouping/grouped_subreddit_data/quarterly_statistics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly counts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run info" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Quarterly counts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Run info" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,22 +460,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>88</v>
+        <v>15</v>
       </c>
       <c r="C2" t="n">
-        <v>486</v>
+        <v>95</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>221</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>146</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -485,22 +485,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>163</v>
+        <v>31</v>
       </c>
       <c r="C3" t="n">
-        <v>741</v>
+        <v>157</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>270</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>222</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -510,22 +510,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>343</v>
+        <v>62</v>
       </c>
       <c r="C4" t="n">
-        <v>1289</v>
+        <v>259</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>293</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>371</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>510</v>
+        <v>62</v>
       </c>
       <c r="C5" t="n">
-        <v>1449</v>
+        <v>334</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>384</v>
+        <v>7</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>520</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6">
@@ -560,22 +560,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>734</v>
+        <v>89</v>
       </c>
       <c r="C6" t="n">
-        <v>1835</v>
+        <v>417</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>505</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>617</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7">
@@ -585,22 +585,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>873</v>
+        <v>99</v>
       </c>
       <c r="C7" t="n">
-        <v>2320</v>
+        <v>536</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>612</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>770</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8">
@@ -610,22 +610,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1590</v>
+        <v>239</v>
       </c>
       <c r="C8" t="n">
-        <v>2913</v>
+        <v>691</v>
       </c>
       <c r="D8" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E8" t="n">
-        <v>544</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>1064</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9">
@@ -635,22 +635,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1857</v>
+        <v>280</v>
       </c>
       <c r="C9" t="n">
-        <v>3365</v>
+        <v>817</v>
       </c>
       <c r="D9" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E9" t="n">
-        <v>798</v>
+        <v>14</v>
       </c>
       <c r="F9" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1262</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10">
@@ -713,7 +713,7 @@
         <v>323</v>
       </c>
       <c r="C12" t="n">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="D12" t="n">
         <v>15</v>
@@ -725,7 +725,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -738,7 +738,7 @@
         <v>435</v>
       </c>
       <c r="C13" t="n">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D13" t="n">
         <v>31</v>
@@ -750,7 +750,7 @@
         <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14">
@@ -763,7 +763,7 @@
         <v>721</v>
       </c>
       <c r="C14" t="n">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="D14" t="n">
         <v>6</v>
@@ -788,7 +788,7 @@
         <v>1190</v>
       </c>
       <c r="C15" t="n">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="D15" t="n">
         <v>8</v>
@@ -800,7 +800,7 @@
         <v>50</v>
       </c>
       <c r="G15" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -813,7 +813,7 @@
         <v>1637</v>
       </c>
       <c r="C16" t="n">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="D16" t="n">
         <v>12</v>
@@ -825,7 +825,7 @@
         <v>64</v>
       </c>
       <c r="G16" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
@@ -838,7 +838,7 @@
         <v>1892</v>
       </c>
       <c r="C17" t="n">
-        <v>1188</v>
+        <v>1184</v>
       </c>
       <c r="D17" t="n">
         <v>10</v>
@@ -863,7 +863,7 @@
         <v>2400</v>
       </c>
       <c r="C18" t="n">
-        <v>1382</v>
+        <v>1374</v>
       </c>
       <c r="D18" t="n">
         <v>5</v>
@@ -875,7 +875,7 @@
         <v>118</v>
       </c>
       <c r="G18" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19">
@@ -888,7 +888,7 @@
         <v>2118</v>
       </c>
       <c r="C19" t="n">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="D19" t="n">
         <v>3</v>
@@ -900,7 +900,7 @@
         <v>145</v>
       </c>
       <c r="G19" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20">
@@ -913,7 +913,7 @@
         <v>2133</v>
       </c>
       <c r="C20" t="n">
-        <v>1377</v>
+        <v>1372</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
@@ -938,7 +938,7 @@
         <v>1805</v>
       </c>
       <c r="C21" t="n">
-        <v>1409</v>
+        <v>1398</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -950,7 +950,7 @@
         <v>230</v>
       </c>
       <c r="G21" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22">
@@ -963,7 +963,7 @@
         <v>1635</v>
       </c>
       <c r="C22" t="n">
-        <v>1458</v>
+        <v>1448</v>
       </c>
       <c r="D22" t="n">
         <v>4</v>
@@ -975,7 +975,7 @@
         <v>252</v>
       </c>
       <c r="G22" t="n">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23">
@@ -988,7 +988,7 @@
         <v>1428</v>
       </c>
       <c r="C23" t="n">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="D23" t="n">
         <v>4</v>
@@ -1013,7 +1013,7 @@
         <v>1502</v>
       </c>
       <c r="C24" t="n">
-        <v>1257</v>
+        <v>1259</v>
       </c>
       <c r="D24" t="n">
         <v>9</v>
@@ -1025,7 +1025,7 @@
         <v>233</v>
       </c>
       <c r="G24" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25">
@@ -1050,7 +1050,7 @@
         <v>284</v>
       </c>
       <c r="G25" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="26">
@@ -1063,7 +1063,7 @@
         <v>1367</v>
       </c>
       <c r="C26" t="n">
-        <v>1215</v>
+        <v>1217</v>
       </c>
       <c r="D26" t="n">
         <v>28</v>
@@ -1075,7 +1075,7 @@
         <v>258</v>
       </c>
       <c r="G26" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="27">
@@ -1088,7 +1088,7 @@
         <v>1287</v>
       </c>
       <c r="C27" t="n">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="D27" t="n">
         <v>14</v>
@@ -1113,7 +1113,7 @@
         <v>1333</v>
       </c>
       <c r="C28" t="n">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="D28" t="n">
         <v>7</v>
@@ -1188,7 +1188,7 @@
         <v>913</v>
       </c>
       <c r="C31" t="n">
-        <v>907</v>
+        <v>904</v>
       </c>
       <c r="D31" t="n">
         <v>16</v>
@@ -1275,7 +1275,7 @@
         <v>201</v>
       </c>
       <c r="G34" t="n">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="35">
@@ -1285,10 +1285,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C35" t="n">
-        <v>763</v>
+        <v>758</v>
       </c>
       <c r="D35" t="n">
         <v>45</v>
@@ -1300,7 +1300,7 @@
         <v>286</v>
       </c>
       <c r="G35" t="n">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="36">
@@ -1313,7 +1313,7 @@
         <v>850</v>
       </c>
       <c r="C36" t="n">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="D36" t="n">
         <v>49</v>
@@ -1325,7 +1325,7 @@
         <v>318</v>
       </c>
       <c r="G36" t="n">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="37">
@@ -1335,10 +1335,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="C37" t="n">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="D37" t="n">
         <v>67</v>
@@ -1360,10 +1360,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>934</v>
+        <v>927</v>
       </c>
       <c r="C38" t="n">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="D38" t="n">
         <v>49</v>
@@ -1375,7 +1375,7 @@
         <v>274</v>
       </c>
       <c r="G38" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="39">
@@ -1388,7 +1388,7 @@
         <v>890</v>
       </c>
       <c r="C39" t="n">
-        <v>2485</v>
+        <v>2484</v>
       </c>
       <c r="D39" t="n">
         <v>50</v>
@@ -1410,10 +1410,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="C40" t="n">
-        <v>3273</v>
+        <v>3271</v>
       </c>
       <c r="D40" t="n">
         <v>79</v>
@@ -1435,10 +1435,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="C41" t="n">
-        <v>2411</v>
+        <v>2410</v>
       </c>
       <c r="D41" t="n">
         <v>104</v>
@@ -1463,7 +1463,7 @@
         <v>1139</v>
       </c>
       <c r="C42" t="n">
-        <v>1915</v>
+        <v>1914</v>
       </c>
       <c r="D42" t="n">
         <v>133</v>
@@ -1475,7 +1475,7 @@
         <v>243</v>
       </c>
       <c r="G42" t="n">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="43">
@@ -1500,7 +1500,7 @@
         <v>87</v>
       </c>
       <c r="G43" t="n">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="44">
@@ -1525,7 +1525,7 @@
         <v>45</v>
       </c>
       <c r="G44" t="n">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="45">
@@ -1538,7 +1538,7 @@
         <v>1011</v>
       </c>
       <c r="C45" t="n">
-        <v>1336</v>
+        <v>1312</v>
       </c>
       <c r="D45" t="n">
         <v>275</v>
@@ -1550,7 +1550,7 @@
         <v>38</v>
       </c>
       <c r="G45" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="46">
@@ -1563,7 +1563,7 @@
         <v>903</v>
       </c>
       <c r="C46" t="n">
-        <v>1863</v>
+        <v>1846</v>
       </c>
       <c r="D46" t="n">
         <v>144</v>
@@ -1575,7 +1575,7 @@
         <v>26</v>
       </c>
       <c r="G46" t="n">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="47">
@@ -1588,7 +1588,7 @@
         <v>1010</v>
       </c>
       <c r="C47" t="n">
-        <v>1823</v>
+        <v>1810</v>
       </c>
       <c r="D47" t="n">
         <v>135</v>
@@ -1600,7 +1600,7 @@
         <v>36</v>
       </c>
       <c r="G47" t="n">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="48">
@@ -1610,10 +1610,10 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="C48" t="n">
-        <v>2200</v>
+        <v>2175</v>
       </c>
       <c r="D48" t="n">
         <v>111</v>
@@ -1625,7 +1625,7 @@
         <v>46</v>
       </c>
       <c r="G48" t="n">
-        <v>442</v>
+        <v>436</v>
       </c>
     </row>
   </sheetData>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:23</t>
+          <t>2026-10-17T21:56:18</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0h 16m 35s</t>
+          <t>0h 08m 15s</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0h 16m 40s</t>
+          <t>0h 08m 17s</t>
         </is>
       </c>
     </row>

</xml_diff>